<commit_message>
feat: migrar indicadores rh para leitura via excel
</commit_message>
<xml_diff>
--- a/data/Indicadores_Compras_Fornecedores/INDICADOR_PROVEDORES.xlsx
+++ b/data/Indicadores_Compras_Fornecedores/INDICADOR_PROVEDORES.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eduar\Downloads\aps-producao\data\Indicadores_Compras_Fornecedores\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19ABB1D8-A920-4E40-BEEA-70945E6716DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{043AC60A-FA16-46AE-9071-4C98534EA440}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{043AC60A-FA16-46AE-9071-4C98534EA440}"/>
   </bookViews>
   <sheets>
     <sheet name="ENTREGAS PROVEDOR EXT. NO PRAZO" sheetId="1" r:id="rId1"/>

</xml_diff>